<commit_message>
he quitado la pestaña objetivos
</commit_message>
<xml_diff>
--- a/informes/informe_seguimiento_alberto_martinez.xlsx
+++ b/informes/informe_seguimiento_alberto_martinez.xlsx
@@ -11,7 +11,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mar 20261" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abr 2026" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evolución" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Objetivos" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -93,7 +92,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -118,16 +117,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D4EDDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EAF7EE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDECEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,7 +146,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -232,18 +221,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1878,254 +1855,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>Objetivos y umbrales de referencia</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Métrica</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>Referencia</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>Positivo si...</t>
-        </is>
-      </c>
-      <c r="D3" s="17" t="inlineStr">
-        <is>
-          <t>Mejorar si...</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>Desgaste total</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>&gt;200 pts</t>
-        </is>
-      </c>
-      <c r="C4" s="28" t="inlineStr">
-        <is>
-          <t>≥200 pts</t>
-        </is>
-      </c>
-      <c r="D4" s="29" t="inlineStr">
-        <is>
-          <t>&lt;200 pts — seguimiento prioritario</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
-        <is>
-          <t>CAL1SEM</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>≥5,0</t>
-        </is>
-      </c>
-      <c r="C5" s="28" t="inlineStr">
-        <is>
-          <t>≥5,0</t>
-        </is>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
-        <is>
-          <t>&lt;5,0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
-        <is>
-          <t>Full/Long Drive</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Media equipo: 11,1 ops</t>
-        </is>
-      </c>
-      <c r="C6" s="28" t="inlineStr">
-        <is>
-          <t>&gt;11,1 ops</t>
-        </is>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>≤11,1 ops</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
-        <is>
-          <t>Fidelidad</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Media equipo: 63,48%</t>
-        </is>
-      </c>
-      <c r="C7" s="28" t="inlineStr">
-        <is>
-          <t>≥63,48%</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>&lt;63,48%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
-        <is>
-          <t>Horch Lauden (pos)</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>≤50 aceptable</t>
-        </is>
-      </c>
-      <c r="C8" s="28" t="inlineStr">
-        <is>
-          <t>≤20 dest. / ≤50 acept.</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>&gt;50 — requiere atención</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
-        <is>
-          <t>ONE Score SEM</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Por encima de la media (6,2)</t>
-        </is>
-      </c>
-      <c r="C9" s="28" t="inlineStr">
-        <is>
-          <t>&gt;6,2</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>≤6,2</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
-        <is>
-          <t>ONE Service CAM</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>≥8%</t>
-        </is>
-      </c>
-      <c r="C10" s="28" t="inlineStr">
-        <is>
-          <t>≥8%</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>5-8% regular / &lt;5% mejorar</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
-        <is>
-          <t>ONE Diferidos</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>≥8%</t>
-        </is>
-      </c>
-      <c r="C11" s="28" t="inlineStr">
-        <is>
-          <t>≥8%</t>
-        </is>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>5-8% regular / &lt;5% mejorar</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="27" t="inlineStr">
-        <is>
-          <t>ONE Multimedia</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>≥5</t>
-        </is>
-      </c>
-      <c r="C12" s="28" t="inlineStr">
-        <is>
-          <t>≥5</t>
-        </is>
-      </c>
-      <c r="D12" s="29" t="inlineStr">
-        <is>
-          <t>3-5 regular / &lt;3 mejorar</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
he metido la calidad de abril
</commit_message>
<xml_diff>
--- a/informes/informe_seguimiento_alberto_martinez.xlsx
+++ b/informes/informe_seguimiento_alberto_martinez.xlsx
@@ -1057,7 +1057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1272,207 +1272,267 @@
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>Sin datos registrados</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>PUNTOS POSITIVOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Satisfacción General (CEM Q4): 4,91 — 2/2 pts  |  Referencia: 0pts &lt;4,60 | 1pt ≥4,60 | 2pts ≥4,80</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Medidas de Servicio (EC28): 0,00% — 2/2 pts  |  Referencia: 0pts &gt;5% | 1pt ≤5% | 2pts ≤1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Conectividad Posventa: 47,30% — 2/2 pts  |  Referencia: 0pts &lt;25% | 1pt ≥25% | 2pts ≥45%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>PUNTOS A MEJORAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Información Proceso (TRS): 82,61% — 1/2 pts  |  Referencia: 0pts &lt;80% | 1pt ≥80% | 2pts ≥90%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>8. ONE KVPS</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>PUNTOS POSITIVOS</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B36" s="7" t="inlineStr">
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Instalación ONE: Asesor</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>Score SEM: 6,3 (media equipo: 6,2) — por encima de la media</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Multimedia Acum.: 5,3 (media equipo: 6,1; bueno ≥5) — en rango positivo</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>PUNTOS A MEJORAR</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="inlineStr">
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Service CAM Acum.: 0% (media equipo: 8%; bueno ≥8%) — por debajo del objetivo</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
+    <row r="46" ht="28" customHeight="1">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="inlineStr">
         <is>
           <t>Diferidos Acum.: 2% (media equipo: 16%; bueno ≥8%) — por debajo del objetivo</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>9. Tareas pendientes</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="12" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t>Tarea</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="C44" s="12" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>Fecha límite</t>
         </is>
       </c>
-      <c r="D44" s="12" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
       </c>
-      <c r="E44" s="12" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>Grado de cumplimentación</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Utilizar el Laser de desgaste</t>
         </is>
       </c>
-      <c r="B45" s="13" t="inlineStr"/>
-      <c r="C45" s="13" t="inlineStr"/>
-      <c r="D45" s="13" t="inlineStr"/>
-      <c r="E45" s="13" t="inlineStr"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="B50" s="13" t="inlineStr"/>
+      <c r="C50" s="13" t="inlineStr"/>
+      <c r="D50" s="13" t="inlineStr"/>
+      <c r="E50" s="13" t="inlineStr"/>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>Full drive</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr"/>
-      <c r="C46" s="14" t="inlineStr"/>
-      <c r="D46" s="14" t="inlineStr"/>
-      <c r="E46" s="14" t="inlineStr"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="B51" s="14" t="inlineStr"/>
+      <c r="C51" s="14" t="inlineStr"/>
+      <c r="D51" s="14" t="inlineStr"/>
+      <c r="E51" s="14" t="inlineStr"/>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="13" t="inlineStr">
         <is>
           <t>Mirar condiciones de la copa horch. Esta en el portal interno</t>
         </is>
       </c>
-      <c r="B47" s="13" t="inlineStr"/>
-      <c r="C47" s="13" t="inlineStr"/>
-      <c r="D47" s="13" t="inlineStr"/>
-      <c r="E47" s="13" t="inlineStr"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="14" t="inlineStr">
+      <c r="B52" s="13" t="inlineStr"/>
+      <c r="C52" s="13" t="inlineStr"/>
+      <c r="D52" s="13" t="inlineStr"/>
+      <c r="E52" s="13" t="inlineStr"/>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>Kpis de one arriba indicados.</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr"/>
-      <c r="C48" s="14" t="inlineStr"/>
-      <c r="D48" s="14" t="inlineStr"/>
-      <c r="E48" s="14" t="inlineStr"/>
+      <c r="B53" s="14" t="inlineStr"/>
+      <c r="C53" s="14" t="inlineStr"/>
+      <c r="D53" s="14" t="inlineStr"/>
+      <c r="E53" s="14" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="39">
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="B46:F46"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B43:F43"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="A32:F32"/>
+    <mergeCell ref="B42:F42"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A17:F17"/>
-    <mergeCell ref="A35:F35"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="A43:F43"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A28:F28"/>
-    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="A44:F44"/>
     <mergeCell ref="B19:F19"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="B37:F37"/>
-    <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A48:F48"/>
     <mergeCell ref="A39:F39"/>
-    <mergeCell ref="B40:F40"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="B33:F33"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B45:F45"/>
     <mergeCell ref="B41:F41"/>
     <mergeCell ref="A25:F25"/>
+    <mergeCell ref="B35:F35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1741,10 +1801,8 @@
       <c r="B20" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="C20" s="21" t="n">
+        <v>7</v>
       </c>
       <c r="D20" s="22" t="inlineStr">
         <is>

</xml_diff>